<commit_message>
Use Czech descriptions in ACO Marine HS summary
Replace the Description column with the sender-supplied Czech names
(Vakuova pumpa, Dmychadlo, Odstrediva pumpa, Provzdusnovaci elementy,
Acidic - MSDS v priloze, Paleta) per the Czech-prioritised rule, keeping
the English name in brackets for reference.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CoFh4Bovwxy5eZWScMyamj
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_ACO_Marine_9280001069.xlsx
+++ b/output/HS_Code_Summary_ACO_Marine_9280001069.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Vacuum pump WVSP R25, 400-460V</t>
+          <t>Vakuová pumpa (Vacuum pump WVSP R25, 400-460V)</t>
         </is>
       </c>
       <c r="C9" s="8" t="n">
@@ -665,7 +665,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Blower SV201/1 2,20kW</t>
+          <t>Dmychadlo (Blower SV201/1 2,20kW)</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
@@ -699,7 +699,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Desludge pump NGA 1B 220/440V/60Hz</t>
+          <t>Odstředivá pumpa (Desludge pump NGA 1B 220/440V/60Hz)</t>
         </is>
       </c>
       <c r="C11" s="8" t="n">
@@ -733,7 +733,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Aeration element L=650 + L=750 (2 line items merged)</t>
+          <t>Provzdušňovací elementy (Aeration element L=650 + L=750, 2 line items merged)</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
@@ -767,7 +767,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>ACO Memcleaner Acidic, 25 l barrel</t>
+          <t>Acidic – MSDS v příloze (ACO Memcleaner Acidic, 25 l barrel)</t>
         </is>
       </c>
       <c r="C13" s="8" t="n">
@@ -801,7 +801,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Europallet 800x1200 (wooden pallet)</t>
+          <t>Paleta (Europallet 800x1200, wooden pallet)</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
@@ -902,7 +902,7 @@
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="19" t="inlineStr">
         <is>
-          <t>NOTE - Description language: The source documents contain English item descriptions only; no Czech descriptions were available, so English is used per the fallback rule.</t>
+          <t>NOTE - Description language: Czech descriptions supplied by the sender are used as the primary description (Czech prioritised per the standing rule), with the original English item name kept in brackets for reference.</t>
         </is>
       </c>
     </row>

</xml_diff>